<commit_message>
Update soccer trades 2026-07-25 13:52:17 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Outrights - World Cup/trades.xlsx
+++ b/data/sxbet/ligas/Outrights - World Cup/trades.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Trades" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,127 +413,216 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:V2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="44" customWidth="1" min="11" max="11"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>gameDate</t>
+          <t>fillHash</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>game</t>
+          <t>bettor</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>side</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>stake</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>odds</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>marketLabel</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>betLabel</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>competition</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>bet</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>market</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>betValue</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>gameLabel</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>teamOneName</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>teamTwoName</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>marketHash</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>sportXeventId</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>maker</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>tradeStatus</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>valid</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
         <is>
           <t>betTime</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>betAmount</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>odds</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>isMarketMaker</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>wallet</t>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>gameTime</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>netReturn</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>chainVersion</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>baseToken</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-22 12:00:00 UTC</t>
+          <t>0x75e09203ba71d6996e0d75dc3aaf36c04fd2c825221e82769d37595c98f267d5</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>0x86821BFbd9111117E4B81a7E6D9e571f80e6A8B5</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>450</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1.9375</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Outright Winner</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>The Field</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Outrights - World Cup</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t>Brazil vs The Field</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Outrights - World Cup</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
         <is>
           <t>The Field</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Outright Winner</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>450</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2026-06-24 15:14:36 UTC</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
-        <v>450</v>
-      </c>
-      <c r="I2" t="n">
-        <v>1.9375</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>0x86821BFbd9111117E4B81a7E6D9e571f80e6A8B5</t>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>0x9fe1daa511ab93bcded3419b8492b0ea750db95b991e0e676042494b11b1b4f8</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>S1781204400:brazil:the-field</t>
+        </is>
+      </c>
+      <c r="N2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R2" t="n">
+        <v>1782314076</v>
+      </c>
+      <c r="S2" t="n">
+        <v>1784721600</v>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>480.0</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>
       </c>
     </row>

</xml_diff>